<commit_message>
US-11148 template xlsx remove parser warning on header/footer
</commit_message>
<xml_diff>
--- a/bin/addons/account/report/account_general_ledger_template.xlsx
+++ b/bin/addons/account/report/account_general_ledger_template.xlsx
@@ -2,12 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13245"/>
   </bookViews>
@@ -1313,9 +1308,5 @@
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="71" orientation="landscape" r:id="rId1"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;"Arial,Bold"&amp;14General Ledger</oddHeader>
-    <oddFooter>Page &amp;P of &amp;N</oddFooter>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>